<commit_message>
feat(skill-assessment): add HR assessment workflow
Includes employee import idempotency, workspace duplicate search tools, and Telegram exam routing/HR notification fixes so copied employee lists and regulation-based exams behave correctly.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/app/data/universal/client_regulations.xlsx
+++ b/app/data/universal/client_regulations.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ТОО\4 dept\4A soft\10A soft\27 Постановка и контроль задача через бота\для_загрузок\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MyActivity\MyInfoBusiness\MyPythonApps\10 Typical_infrastructure\app\data\universal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60E60B57-AEE7-4B0C-8E4A-A0CBA41A3DE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F4B654C-CC0D-4288-AF76-AAEED9AB6C2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="client_regulations" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="192">
   <si>
     <t>id</t>
   </si>
@@ -94,9 +107,6 @@
     <t>ACC</t>
   </si>
   <si>
-    <t>V1</t>
-  </si>
-  <si>
     <t>active</t>
   </si>
   <si>
@@ -442,60 +452,6 @@
     <t>План продаж отдела выполняется в согласованный период не за счёт случайных разовых успехов, а через стабильную систему управления воронкой, людьми, активностями и приоритетами.</t>
   </si>
   <si>
-    <t>https://docs.google.com/document/d/19g0BHFR5tsLIEe7yNpYT_s7HbXJM0SlhWe59mti0-r8/edit?usp=sharing</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/document/d/1yVRoPwXvJEd4QQX-_OLbn95CeiTIrUeNlM8Np70KaKk/edit?usp=drive_link</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/document/d/10wWFvVRSpCdN7zbRQjO6eDpwL55CGCs2qWr8oBM8YZY/edit?usp=drive_link</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/document/d/1F22ISXZyPvIae78D1XgQBV33OpnQnTFdemh7LbkxrRE/edit?usp=drive_link</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/document/d/10Z4PDjFuVL-QSragS-HvsDdNEjxbusTqCt4owg0YI2U/edit?usp=drive_link</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/document/d/15mneHx9sbd0aIDpTV1RvXpKcBvASKieCwkxqn_1WwWo/edit?usp=drive_link</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/document/d/1DE1sg8VouGysvr6uEXZHUB84M6pC5NgNB-dqyLzlWbw/edit?usp=drive_link</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/document/d/14IWi2a8coClYGqatvIjrCZR7A9bkCNsUjl02GtfLz38/edit?usp=drive_link</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/document/d/1EquOj-_b2IFebxOieriwN_s558pN-IzNWrzMr9tQ59A/edit?usp=drive_link</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/document/d/1fPvg88E-JlVPVqf4-BIrGxceADhVFwacOu5Cod4M6yk/edit?usp=drive_link</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/document/d/1myRYfBFv73LbdPwxMNEu9MukxUXkvj_r8WUrPwIQ2VU/edit?usp=drive_link</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/document/d/1P3jkgimNdz5n2Eq6CI4S1pyjYgQWXfL1-BrF48kPNiA/edit?usp=drive_link</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/document/d/1ik2YSFxbfxIc8ryDRYXQ-kJdH2RQ8Ovx23ALQmJW4Cs/edit?usp=drive_link</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/document/d/1yVRoPwXvJEd4QQX-_OLbn95CeiTIrUeNlM8Np70KaKk/edit?usp=sharing</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/document/d/1_my33YP7SrovqfkXP2Tl2EolgPLr0HUfwwcWN-GQvuw/edit?usp=sharing</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/document/d/1s8iE_xOFc8KFsLBM-5YnVGvIuUkYrx6XbGLJnFJLBBk/edit?usp=drive_link</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/document/d/1LvDs4mTPcvc_kEmwO7zV4vlT5zi84wFZ21vTrJgi0Ao/edit?usp=sharing</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/document/d/1cgrftiD59S3zbVYE7ffRq3S2-v8d5m3JoAqn_6RCzUo/edit?usp=sharing</t>
-  </si>
-  <si>
     <t>Управляемая работа компании</t>
   </si>
   <si>
@@ -545,6 +501,114 @@
   </si>
   <si>
     <t>Управляемые внешние коммуникации</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/document/d/1nIlEBtWKOFVzjxqGVwkIQvF0md_1xw7kLMvA5aUa0g0/edit?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/document/d/1kySyFsCmkGJMkmK35iBoHEw5d87YlCDsrndjrOefwZY/edit?usp=sharing</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/document/d/1LFCEevbO8339_xOgECQquZ21Q9kco_v0rJUgQff-Mw8/edit?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/document/d/1T76VDsPJBcH30KQUC1Z3fYizaraiYSltE8uX4gXZ3gE/edit?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/document/d/1jOgPLv6nYbwGcqJ2VfKeLbOCq1C0bTVsE91COjimwAQ/edit?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/document/d/1BxNPYGYQtLED47zaC7iGv9D1YMR4dSO9WxQ7wd1p04Q/edit?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/document/d/1BKnjtODOLHAYyrYnXMl_hHI6lgtjbIouuwr3UyZdPiA/edit?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/document/d/1eUEfbwkLSJ73cpVNMQklV-n3zDQ1vWAtP2Xjku6arLo/edit?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/document/d/1HIUKDVCFi-9AuCM5vVt5ZPU6ysKb_D1Yak6XLeDCAgk/edit?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/document/d/1hNQaDTFfxdDM5MEJS9h4hxHWfrFFGYRDoZMsJeREmVM/edit?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/document/d/1ZiQ1S4SCDXYGgrn7fvkeWVzCvsC_EXIKU0KJPsCb4RQ/edit?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/document/d/1vNTwLOAroBUZFnwZDR33ZGs50-XGH1PalSfdcUxaZPA/edit?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/document/d/1pzz0xeEQOvqupsL7rnKIIp1wd0usVX94lx2xo41uVRQ/edit?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/document/d/15E35tFyim-Dkv6Hp6EnOEmGXk32V9fbDC1Z3_ONNAi8/edit?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/document/d/1cRtOLK6kx71dlDaYoXM_aIaL7RCEq2bX8n7rSv1pd4c/edit?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/document/d/1HrWrhT5qw2GM8_zXkP5rsjtcJmSJ671U3DGwKHF52zY/edit?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/document/d/1ZuWRwpfzyJIb88bFOSh7JEQXeDVsEME4K71xjnTKrBc/edit?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>V2</t>
+  </si>
+  <si>
+    <t>REG_DIRECTOR_V2</t>
+  </si>
+  <si>
+    <t>REG_ADM_ZAMADM_V2</t>
+  </si>
+  <si>
+    <t>REG_PROD_SUPERVISOR_V2</t>
+  </si>
+  <si>
+    <t>REG_HR_HEAD_V2</t>
+  </si>
+  <si>
+    <t>REG_HR_MANAGER_V2</t>
+  </si>
+  <si>
+    <t>REG_HR_RECRUITER_V2</t>
+  </si>
+  <si>
+    <t>REG_SYSADMIN_V2</t>
+  </si>
+  <si>
+    <t>REG_INFO_SYSTEM_SUPPORT_V2</t>
+  </si>
+  <si>
+    <t>REG_LEADGEN_SPECIALIST_V2</t>
+  </si>
+  <si>
+    <t>REG_MKT_MANAGER_V2</t>
+  </si>
+  <si>
+    <t>REG_SALES_MGR_V2</t>
+  </si>
+  <si>
+    <t>REG_SALES_TEAM_LEAD_V2</t>
+  </si>
+  <si>
+    <t>REG_ACC_CHIEF_ACCOUNTANT_V2</t>
+  </si>
+  <si>
+    <t>REG_ACC_MATERIAL_ACCOUNTANT_V2</t>
+  </si>
+  <si>
+    <t>REG_PROD_TECH_DIR_V2</t>
+  </si>
+  <si>
+    <t>REG_QUAL_HEAD_V2</t>
+  </si>
+  <si>
+    <t>REG_QUAL_SPECIALIST_V2</t>
+  </si>
+  <si>
+    <t>REG_PR_SPECIALIST_V2</t>
   </si>
 </sst>
 </file>
@@ -923,8 +987,10 @@
   <dimension ref="A1:V19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="3" max="3" width="41.5546875" customWidth="1"/>
     <col min="6" max="6" width="27" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="14.6640625" customWidth="1"/>
+    <col min="15" max="22" width="2.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.3">
@@ -997,46 +1063,46 @@
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
         <v>22</v>
       </c>
       <c r="C2" t="s">
+        <v>174</v>
+      </c>
+      <c r="D2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
         <v>39</v>
       </c>
-      <c r="D2" t="s">
-        <v>39</v>
-      </c>
-      <c r="E2" t="b">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>40</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>41</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>42</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="K2" t="s">
         <v>43</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="L2" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="K2" t="s">
-        <v>44</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>140</v>
-      </c>
       <c r="N2" t="s">
+        <v>173</v>
+      </c>
+      <c r="O2" t="s">
         <v>24</v>
-      </c>
-      <c r="O2" t="s">
-        <v>25</v>
       </c>
       <c r="R2" t="b">
         <v>1</v>
@@ -1050,46 +1116,46 @@
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B3" t="s">
         <v>22</v>
       </c>
       <c r="C3" t="s">
+        <v>175</v>
+      </c>
+      <c r="D3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
         <v>52</v>
       </c>
-      <c r="D3" t="s">
-        <v>52</v>
-      </c>
-      <c r="E3" t="b">
-        <v>1</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H3" t="s">
         <v>53</v>
       </c>
-      <c r="G3" t="s">
-        <v>41</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>54</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="K3" t="s">
         <v>55</v>
       </c>
-      <c r="J3" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="K3" t="s">
-        <v>56</v>
-      </c>
       <c r="L3" s="2" t="s">
-        <v>142</v>
+        <v>160</v>
       </c>
       <c r="N3" t="s">
+        <v>173</v>
+      </c>
+      <c r="O3" t="s">
         <v>24</v>
-      </c>
-      <c r="O3" t="s">
-        <v>25</v>
       </c>
       <c r="R3" t="b">
         <v>1</v>
@@ -1103,46 +1169,46 @@
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B4" t="s">
         <v>22</v>
       </c>
       <c r="C4" t="s">
+        <v>176</v>
+      </c>
+      <c r="D4" t="s">
+        <v>96</v>
+      </c>
+      <c r="E4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F4" t="s">
         <v>97</v>
       </c>
-      <c r="D4" t="s">
-        <v>97</v>
-      </c>
-      <c r="E4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>98</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>99</v>
       </c>
-      <c r="H4" t="s">
-        <v>100</v>
-      </c>
       <c r="I4" t="s">
+        <v>104</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="K4" t="s">
         <v>105</v>
       </c>
-      <c r="J4" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="K4" t="s">
-        <v>106</v>
-      </c>
       <c r="L4" s="2" t="s">
-        <v>141</v>
+        <v>167</v>
       </c>
       <c r="N4" t="s">
+        <v>173</v>
+      </c>
+      <c r="O4" t="s">
         <v>24</v>
-      </c>
-      <c r="O4" t="s">
-        <v>25</v>
       </c>
       <c r="R4" t="b">
         <v>1</v>
@@ -1156,46 +1222,46 @@
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B5" t="s">
         <v>22</v>
       </c>
       <c r="C5" t="s">
+        <v>177</v>
+      </c>
+      <c r="D5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s">
         <v>59</v>
       </c>
-      <c r="D5" t="s">
-        <v>59</v>
-      </c>
-      <c r="E5" t="b">
-        <v>1</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
+        <v>56</v>
+      </c>
+      <c r="H5" t="s">
         <v>60</v>
       </c>
-      <c r="G5" t="s">
-        <v>57</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>61</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="K5" t="s">
         <v>62</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="L5" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="K5" t="s">
-        <v>63</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>154</v>
-      </c>
       <c r="N5" t="s">
+        <v>173</v>
+      </c>
+      <c r="O5" t="s">
         <v>24</v>
-      </c>
-      <c r="O5" t="s">
-        <v>25</v>
       </c>
       <c r="R5" t="b">
         <v>1</v>
@@ -1209,46 +1275,46 @@
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B6" t="s">
         <v>22</v>
       </c>
       <c r="C6" t="s">
+        <v>178</v>
+      </c>
+      <c r="D6" t="s">
+        <v>64</v>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" t="s">
         <v>65</v>
       </c>
-      <c r="D6" t="s">
-        <v>65</v>
-      </c>
-      <c r="E6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H6" t="s">
         <v>66</v>
       </c>
-      <c r="G6" t="s">
-        <v>57</v>
-      </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>67</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="K6" t="s">
         <v>68</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="L6" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="K6" t="s">
-        <v>69</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>145</v>
-      </c>
       <c r="N6" t="s">
+        <v>173</v>
+      </c>
+      <c r="O6" t="s">
         <v>24</v>
-      </c>
-      <c r="O6" t="s">
-        <v>25</v>
       </c>
       <c r="R6" t="b">
         <v>1</v>
@@ -1262,46 +1328,46 @@
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B7" t="s">
         <v>22</v>
       </c>
       <c r="C7" t="s">
+        <v>179</v>
+      </c>
+      <c r="D7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E7" t="b">
+        <v>1</v>
+      </c>
+      <c r="F7" t="s">
         <v>71</v>
       </c>
-      <c r="D7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E7" t="b">
-        <v>1</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H7" t="s">
         <v>72</v>
       </c>
-      <c r="G7" t="s">
-        <v>57</v>
-      </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>73</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="K7" t="s">
         <v>74</v>
       </c>
-      <c r="J7" s="4" t="s">
+      <c r="L7" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="K7" t="s">
-        <v>75</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>144</v>
-      </c>
       <c r="N7" t="s">
+        <v>173</v>
+      </c>
+      <c r="O7" t="s">
         <v>24</v>
-      </c>
-      <c r="O7" t="s">
-        <v>25</v>
       </c>
       <c r="R7" t="b">
         <v>1</v>
@@ -1315,46 +1381,46 @@
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B8" t="s">
         <v>22</v>
       </c>
       <c r="C8" t="s">
+        <v>180</v>
+      </c>
+      <c r="D8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E8" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" t="s">
         <v>46</v>
       </c>
-      <c r="D8" t="s">
-        <v>46</v>
-      </c>
-      <c r="E8" t="b">
-        <v>1</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
+        <v>40</v>
+      </c>
+      <c r="H8" t="s">
         <v>47</v>
       </c>
-      <c r="G8" t="s">
-        <v>41</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>48</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="K8" t="s">
         <v>49</v>
       </c>
-      <c r="J8" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="K8" t="s">
-        <v>50</v>
-      </c>
       <c r="L8" s="2" t="s">
-        <v>146</v>
+        <v>159</v>
       </c>
       <c r="N8" t="s">
+        <v>173</v>
+      </c>
+      <c r="O8" t="s">
         <v>24</v>
-      </c>
-      <c r="O8" t="s">
-        <v>25</v>
       </c>
       <c r="R8" t="b">
         <v>1</v>
@@ -1368,46 +1434,46 @@
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B9" t="s">
         <v>22</v>
       </c>
       <c r="C9" t="s">
+        <v>181</v>
+      </c>
+      <c r="D9" t="s">
+        <v>76</v>
+      </c>
+      <c r="E9" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" t="s">
         <v>77</v>
       </c>
-      <c r="D9" t="s">
-        <v>77</v>
-      </c>
-      <c r="E9" t="b">
-        <v>1</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
+        <v>40</v>
+      </c>
+      <c r="H9" t="s">
         <v>78</v>
       </c>
-      <c r="G9" t="s">
-        <v>41</v>
-      </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>79</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="K9" t="s">
         <v>80</v>
       </c>
-      <c r="J9" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="K9" t="s">
-        <v>81</v>
-      </c>
       <c r="L9" s="2" t="s">
-        <v>147</v>
+        <v>164</v>
       </c>
       <c r="N9" t="s">
+        <v>173</v>
+      </c>
+      <c r="O9" t="s">
         <v>24</v>
-      </c>
-      <c r="O9" t="s">
-        <v>25</v>
       </c>
       <c r="R9" t="b">
         <v>1</v>
@@ -1421,46 +1487,46 @@
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B10" t="s">
         <v>22</v>
       </c>
       <c r="C10" t="s">
+        <v>182</v>
+      </c>
+      <c r="D10" t="s">
+        <v>82</v>
+      </c>
+      <c r="E10" t="b">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s">
         <v>83</v>
       </c>
-      <c r="D10" t="s">
-        <v>83</v>
-      </c>
-      <c r="E10" t="b">
-        <v>1</v>
-      </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>84</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>85</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>86</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="K10" t="s">
         <v>87</v>
       </c>
-      <c r="J10" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="K10" t="s">
-        <v>88</v>
-      </c>
       <c r="L10" s="2" t="s">
-        <v>149</v>
+        <v>165</v>
       </c>
       <c r="N10" t="s">
+        <v>173</v>
+      </c>
+      <c r="O10" t="s">
         <v>24</v>
-      </c>
-      <c r="O10" t="s">
-        <v>25</v>
       </c>
       <c r="R10" t="b">
         <v>1</v>
@@ -1474,46 +1540,46 @@
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B11" t="s">
         <v>22</v>
       </c>
       <c r="C11" t="s">
+        <v>183</v>
+      </c>
+      <c r="D11" t="s">
+        <v>89</v>
+      </c>
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" t="s">
         <v>90</v>
       </c>
-      <c r="D11" t="s">
-        <v>90</v>
-      </c>
-      <c r="E11" t="b">
-        <v>1</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>91</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>92</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>93</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="K11" t="s">
         <v>94</v>
       </c>
-      <c r="J11" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="K11" t="s">
-        <v>95</v>
-      </c>
       <c r="L11" s="2" t="s">
-        <v>148</v>
+        <v>166</v>
       </c>
       <c r="N11" t="s">
+        <v>173</v>
+      </c>
+      <c r="O11" t="s">
         <v>24</v>
-      </c>
-      <c r="O11" t="s">
-        <v>25</v>
       </c>
       <c r="R11" t="b">
         <v>1</v>
@@ -1527,46 +1593,46 @@
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B12" t="s">
         <v>22</v>
       </c>
       <c r="C12" t="s">
+        <v>184</v>
+      </c>
+      <c r="D12" t="s">
+        <v>127</v>
+      </c>
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s">
         <v>128</v>
       </c>
-      <c r="D12" t="s">
-        <v>128</v>
-      </c>
-      <c r="E12" t="b">
-        <v>1</v>
-      </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>129</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>130</v>
       </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>131</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="K12" t="s">
         <v>132</v>
       </c>
-      <c r="J12" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="K12" t="s">
-        <v>133</v>
-      </c>
       <c r="L12" s="2" t="s">
-        <v>151</v>
+        <v>171</v>
       </c>
       <c r="N12" t="s">
+        <v>173</v>
+      </c>
+      <c r="O12" t="s">
         <v>24</v>
-      </c>
-      <c r="O12" t="s">
-        <v>25</v>
       </c>
       <c r="R12" t="b">
         <v>1</v>
@@ -1580,46 +1646,46 @@
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B13" t="s">
         <v>22</v>
       </c>
       <c r="C13" t="s">
+        <v>185</v>
+      </c>
+      <c r="D13" t="s">
+        <v>134</v>
+      </c>
+      <c r="E13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F13" t="s">
         <v>135</v>
       </c>
-      <c r="D13" t="s">
-        <v>135</v>
-      </c>
-      <c r="E13" t="b">
-        <v>1</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
+        <v>129</v>
+      </c>
+      <c r="H13" t="s">
         <v>136</v>
       </c>
-      <c r="G13" t="s">
-        <v>130</v>
-      </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>137</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="K13" t="s">
         <v>138</v>
       </c>
-      <c r="J13" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="K13" t="s">
-        <v>139</v>
-      </c>
       <c r="L13" s="2" t="s">
-        <v>150</v>
+        <v>172</v>
       </c>
       <c r="N13" t="s">
+        <v>173</v>
+      </c>
+      <c r="O13" t="s">
         <v>24</v>
-      </c>
-      <c r="O13" t="s">
-        <v>25</v>
       </c>
       <c r="R13" t="b">
         <v>1</v>
@@ -1633,46 +1699,46 @@
     </row>
     <row r="14" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B14" t="s">
         <v>22</v>
       </c>
       <c r="C14" t="s">
+        <v>186</v>
+      </c>
+      <c r="D14" t="s">
+        <v>26</v>
+      </c>
+      <c r="E14" t="b">
+        <v>1</v>
+      </c>
+      <c r="F14" t="s">
         <v>27</v>
-      </c>
-      <c r="D14" t="s">
-        <v>27</v>
-      </c>
-      <c r="E14" t="b">
-        <v>1</v>
-      </c>
-      <c r="F14" t="s">
-        <v>28</v>
       </c>
       <c r="G14" t="s">
         <v>23</v>
       </c>
       <c r="H14" t="s">
+        <v>28</v>
+      </c>
+      <c r="I14" t="s">
         <v>29</v>
       </c>
-      <c r="I14" t="s">
+      <c r="J14" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="K14" t="s">
         <v>30</v>
       </c>
-      <c r="J14" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="K14" t="s">
-        <v>31</v>
-      </c>
       <c r="L14" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="N14" t="s">
+        <v>173</v>
+      </c>
+      <c r="O14" t="s">
         <v>24</v>
-      </c>
-      <c r="O14" t="s">
-        <v>25</v>
       </c>
       <c r="R14" t="b">
         <v>1</v>
@@ -1686,46 +1752,46 @@
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B15" t="s">
         <v>22</v>
       </c>
       <c r="C15" t="s">
+        <v>187</v>
+      </c>
+      <c r="D15" t="s">
+        <v>32</v>
+      </c>
+      <c r="E15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F15" t="s">
         <v>33</v>
-      </c>
-      <c r="D15" t="s">
-        <v>33</v>
-      </c>
-      <c r="E15" t="b">
-        <v>1</v>
-      </c>
-      <c r="F15" t="s">
-        <v>34</v>
       </c>
       <c r="G15" t="s">
         <v>23</v>
       </c>
       <c r="H15" t="s">
+        <v>34</v>
+      </c>
+      <c r="I15" t="s">
         <v>35</v>
       </c>
-      <c r="I15" t="s">
+      <c r="J15" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="K15" t="s">
         <v>36</v>
       </c>
-      <c r="J15" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="K15" t="s">
-        <v>37</v>
-      </c>
       <c r="L15" s="2" t="s">
-        <v>143</v>
+        <v>157</v>
       </c>
       <c r="N15" t="s">
+        <v>173</v>
+      </c>
+      <c r="O15" t="s">
         <v>24</v>
-      </c>
-      <c r="O15" t="s">
-        <v>25</v>
       </c>
       <c r="R15" t="b">
         <v>1</v>
@@ -1739,46 +1805,46 @@
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B16" t="s">
         <v>22</v>
       </c>
       <c r="C16" t="s">
+        <v>188</v>
+      </c>
+      <c r="D16" t="s">
+        <v>101</v>
+      </c>
+      <c r="E16" t="b">
+        <v>1</v>
+      </c>
+      <c r="F16" t="s">
         <v>102</v>
       </c>
-      <c r="D16" t="s">
-        <v>102</v>
-      </c>
-      <c r="E16" t="b">
-        <v>1</v>
-      </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
+        <v>98</v>
+      </c>
+      <c r="H16" t="s">
         <v>103</v>
       </c>
-      <c r="G16" t="s">
-        <v>99</v>
-      </c>
-      <c r="H16" t="s">
+      <c r="I16" t="s">
         <v>104</v>
       </c>
-      <c r="I16" t="s">
+      <c r="J16" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="K16" t="s">
         <v>105</v>
       </c>
-      <c r="J16" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="K16" t="s">
-        <v>106</v>
-      </c>
       <c r="L16" s="2" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="N16" t="s">
+        <v>173</v>
+      </c>
+      <c r="O16" t="s">
         <v>24</v>
-      </c>
-      <c r="O16" t="s">
-        <v>25</v>
       </c>
       <c r="R16" t="b">
         <v>1</v>
@@ -1792,46 +1858,46 @@
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B17" t="s">
         <v>22</v>
       </c>
       <c r="C17" t="s">
+        <v>189</v>
+      </c>
+      <c r="D17" t="s">
+        <v>114</v>
+      </c>
+      <c r="E17" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" t="s">
         <v>115</v>
       </c>
-      <c r="D17" t="s">
-        <v>115</v>
-      </c>
-      <c r="E17" t="b">
-        <v>1</v>
-      </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>116</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>117</v>
       </c>
-      <c r="H17" t="s">
+      <c r="I17" t="s">
         <v>118</v>
       </c>
-      <c r="I17" t="s">
+      <c r="J17" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="K17" t="s">
         <v>119</v>
       </c>
-      <c r="J17" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="K17" t="s">
-        <v>120</v>
-      </c>
       <c r="L17" s="2" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="N17" t="s">
+        <v>173</v>
+      </c>
+      <c r="O17" t="s">
         <v>24</v>
-      </c>
-      <c r="O17" t="s">
-        <v>25</v>
       </c>
       <c r="R17" t="b">
         <v>1</v>
@@ -1845,46 +1911,46 @@
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B18" t="s">
         <v>22</v>
       </c>
       <c r="C18" t="s">
+        <v>190</v>
+      </c>
+      <c r="D18" t="s">
+        <v>121</v>
+      </c>
+      <c r="E18" t="b">
+        <v>1</v>
+      </c>
+      <c r="F18" t="s">
         <v>122</v>
       </c>
-      <c r="D18" t="s">
-        <v>122</v>
-      </c>
-      <c r="E18" t="b">
-        <v>1</v>
-      </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
+        <v>116</v>
+      </c>
+      <c r="H18" t="s">
         <v>123</v>
       </c>
-      <c r="G18" t="s">
-        <v>117</v>
-      </c>
-      <c r="H18" t="s">
+      <c r="I18" t="s">
         <v>124</v>
       </c>
-      <c r="I18" t="s">
+      <c r="J18" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="K18" t="s">
         <v>125</v>
       </c>
-      <c r="J18" s="4" t="s">
+      <c r="L18" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="N18" t="s">
         <v>173</v>
       </c>
-      <c r="K18" t="s">
-        <v>126</v>
-      </c>
-      <c r="L18" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="N18" t="s">
+      <c r="O18" t="s">
         <v>24</v>
-      </c>
-      <c r="O18" t="s">
-        <v>25</v>
       </c>
       <c r="R18" t="b">
         <v>1</v>
@@ -1898,46 +1964,46 @@
     </row>
     <row r="19" spans="1:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B19" t="s">
         <v>22</v>
       </c>
       <c r="C19" t="s">
+        <v>191</v>
+      </c>
+      <c r="D19" t="s">
+        <v>107</v>
+      </c>
+      <c r="E19" t="b">
+        <v>1</v>
+      </c>
+      <c r="F19" t="s">
         <v>108</v>
       </c>
-      <c r="D19" t="s">
-        <v>108</v>
-      </c>
-      <c r="E19" t="b">
-        <v>1</v>
-      </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>109</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>110</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>111</v>
       </c>
-      <c r="I19" t="s">
+      <c r="J19" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="K19" t="s">
         <v>112</v>
       </c>
-      <c r="J19" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="K19" t="s">
-        <v>113</v>
-      </c>
       <c r="L19" s="2" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="N19" t="s">
+        <v>173</v>
+      </c>
+      <c r="O19" t="s">
         <v>24</v>
-      </c>
-      <c r="O19" t="s">
-        <v>25</v>
       </c>
       <c r="R19" t="b">
         <v>1</v>
@@ -1951,24 +2017,24 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="L2" r:id="rId1" xr:uid="{52021DEB-B498-4F82-8133-C95FEC1A6E58}"/>
-    <hyperlink ref="L4" r:id="rId2" xr:uid="{0D97F35E-2601-46D1-B37A-2133BF0995A9}"/>
-    <hyperlink ref="L7" r:id="rId3" xr:uid="{B5B63096-10F4-49F8-8F3F-750ED7877675}"/>
-    <hyperlink ref="L6" r:id="rId4" xr:uid="{1017E556-779A-4267-A384-00A818B835DB}"/>
-    <hyperlink ref="L8" r:id="rId5" xr:uid="{0131D4D7-7C05-462D-AC06-DA0275165D46}"/>
-    <hyperlink ref="L11" r:id="rId6" xr:uid="{A832D6C7-E3BA-4F20-BB7B-0DCC6AB39A01}"/>
-    <hyperlink ref="L9" r:id="rId7" xr:uid="{1ADD4412-CA16-4519-ADB4-4FF90AD314C8}"/>
-    <hyperlink ref="L13" r:id="rId8" xr:uid="{7C83AB80-41E5-48C0-A442-4282586EC488}"/>
-    <hyperlink ref="L10" r:id="rId9" xr:uid="{1B6915D6-1DD3-4C8E-ADE5-50DE1DD854D6}"/>
-    <hyperlink ref="L15" r:id="rId10" xr:uid="{1F0D3B7D-974D-4189-BC34-3E5948C350DB}"/>
-    <hyperlink ref="L16" r:id="rId11" xr:uid="{B48C2C98-B8B6-41C1-82C5-1B5BCB7F8271}"/>
-    <hyperlink ref="L18" r:id="rId12" xr:uid="{1AE79AE7-B54F-4C37-9932-C59D12B275FD}"/>
-    <hyperlink ref="L3" r:id="rId13" xr:uid="{228B2B36-9E74-4AE4-BDBA-DB2D27BB4734}"/>
-    <hyperlink ref="L5" r:id="rId14" xr:uid="{EC36B77F-2C16-4197-83D4-DB454EA040A5}"/>
-    <hyperlink ref="L12" r:id="rId15" xr:uid="{0E15F45A-DC46-450D-B4C3-0F9038BE2EB1}"/>
-    <hyperlink ref="L14" r:id="rId16" xr:uid="{90DDB8F5-CDA1-4B84-AF36-CE50A642115E}"/>
-    <hyperlink ref="L17" r:id="rId17" xr:uid="{1DC910E9-7609-4E10-AE73-467976F2D68C}"/>
-    <hyperlink ref="L19" r:id="rId18" xr:uid="{6A4570E2-747B-4378-BF91-54EAB130A8BB}"/>
+    <hyperlink ref="L2" r:id="rId1" xr:uid="{5E568F36-8999-42D5-A2B1-876A5811A41A}"/>
+    <hyperlink ref="L3" r:id="rId2" xr:uid="{590B723C-3157-41E2-ACA7-838CE43198AF}"/>
+    <hyperlink ref="L4" r:id="rId3" xr:uid="{85748D5B-6842-40AF-937E-4607951DD539}"/>
+    <hyperlink ref="L5" r:id="rId4" xr:uid="{AB1176BF-41B9-445A-BB5E-BC204F0C5425}"/>
+    <hyperlink ref="L6" r:id="rId5" xr:uid="{BA8792EB-ACF1-42B0-A731-0F7EFA6D25C3}"/>
+    <hyperlink ref="L7" r:id="rId6" xr:uid="{10820748-C789-4310-9A16-F635979CA3C0}"/>
+    <hyperlink ref="L8" r:id="rId7" xr:uid="{D8AF2EFD-FDDE-48DA-97E7-BF3366A61E7C}"/>
+    <hyperlink ref="L9" r:id="rId8" xr:uid="{02FA9B3F-3D8D-4DAF-A6DC-B66C0F126F6C}"/>
+    <hyperlink ref="L10" r:id="rId9" xr:uid="{8095A414-E12A-413D-96AA-11A84361F55B}"/>
+    <hyperlink ref="L11" r:id="rId10" xr:uid="{EFBBC042-4990-43CC-9ACB-C116442DE03E}"/>
+    <hyperlink ref="L12" r:id="rId11" xr:uid="{DFA91DE9-DEC5-4323-A763-62F0C4497F22}"/>
+    <hyperlink ref="L13" r:id="rId12" xr:uid="{8CCAD7BC-2572-4B7E-B1CB-CE3022D914B3}"/>
+    <hyperlink ref="L14" r:id="rId13" xr:uid="{9679954C-E1E4-45B2-BBAD-A0ACFBF32BFE}"/>
+    <hyperlink ref="L15" r:id="rId14" xr:uid="{EA85C02F-B963-42BF-8A69-40F4E76375A4}"/>
+    <hyperlink ref="L16" r:id="rId15" xr:uid="{6F81D7DC-31F8-4A63-AB96-3D87F1CC5625}"/>
+    <hyperlink ref="L17" r:id="rId16" xr:uid="{4680B422-6208-4968-9E4C-1A33C2C54645}"/>
+    <hyperlink ref="L18" r:id="rId17" xr:uid="{AC6850B2-A195-4262-856A-791B77670B26}"/>
+    <hyperlink ref="L19" r:id="rId18" xr:uid="{530312F8-7E4C-49AC-8EA1-28F0656434E3}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>